<commit_message>
Refactor evidence handling in assessment and maturity model components
- Removed `requiresEvidence` property from questions and adjusted related logic in assessmentQuestionResponses, assessmentResultsExport, and assessmentTour.
- Updated evidence grouping to be based on practices instead of questions in various components including evaluationModel and evidenceUpload.
- Modified UI components to reflect changes in evidence requirements and display.
- Adjusted tests to ensure proper functionality with the new evidence structure and requirements.
- Added new tests for practice evidence review to validate evidence handling without unanswered questions.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/maturity-model-template.xlsx
+++ b/frontend/public/templates/maturity-model-template.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="87">
   <si>
     <t>modelName</t>
   </si>
@@ -112,6 +112,9 @@
     <t>practiceDescription</t>
   </si>
   <si>
+    <t>practiceRequiresEvidence</t>
+  </si>
+  <si>
     <t>P1_PD</t>
   </si>
   <si>
@@ -175,18 +178,36 @@
     <t>questionChoices</t>
   </si>
   <si>
-    <t>questionLikertScaleMax</t>
+    <t>questionScalePointCount</t>
+  </si>
+  <si>
+    <t>questionScaleMinLabel</t>
+  </si>
+  <si>
+    <t>questionScaleMaxLabel</t>
+  </si>
+  <si>
+    <t>questionScaleHighPointIsMaximum</t>
   </si>
   <si>
     <t>questionHelp</t>
   </si>
   <si>
-    <t>questionRequiresEvidence</t>
-  </si>
-  <si>
     <t>questionRequired</t>
   </si>
   <si>
+    <t>questionRangeMin</t>
+  </si>
+  <si>
+    <t>questionRangeMax</t>
+  </si>
+  <si>
+    <t>questionRangeHighValueIsMaximum</t>
+  </si>
+  <si>
+    <t>questionRanges</t>
+  </si>
+  <si>
     <t>Q1_APD</t>
   </si>
   <si>
@@ -232,7 +253,7 @@
     <t>multiple_choice</t>
   </si>
   <si>
-    <t>[{"label":"Initial / ad-hoc","level":1},{"label":"Repeatable","level":2},{"label":"Defined","level":3},{"label":"Managed","level":4},{"label":"Optimizing","level":5}]</t>
+    <t>[{"label":"Initial / ad-hoc","score":0.0,"rawValue":null},{"label":"Repeatable","score":0.25,"rawValue":null},{"label":"Defined","score":0.5,"rawValue":null},{"label":"Managed","score":0.75,"rawValue":null},{"label":"Optimizing","score":1.0,"rawValue":null}]</t>
   </si>
   <si>
     <t>Each option maps to a level number on your scale. Use JSON: array of {label level}.</t>
@@ -465,7 +486,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -484,6 +505,9 @@
       <c r="E1" t="s" s="0">
         <v>30</v>
       </c>
+      <c r="F1" t="s" s="0">
+        <v>31</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
@@ -493,13 +517,16 @@
         <v>16</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="F2" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -510,13 +537,16 @@
         <v>19</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>36</v>
+        <v>37</v>
+      </c>
+      <c r="F3" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -527,13 +557,16 @@
         <v>19</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
+      </c>
+      <c r="F4" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -544,13 +577,16 @@
         <v>22</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>42</v>
+        <v>43</v>
+      </c>
+      <c r="F5" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -561,13 +597,16 @@
         <v>25</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>45</v>
+        <v>46</v>
+      </c>
+      <c r="F6" t="b" s="0">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -577,7 +616,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:S7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -591,34 +630,52 @@
         <v>28</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K1" t="s" s="0">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="L1" t="s" s="0">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="M1" t="s" s="0">
-        <v>55</v>
+        <v>56</v>
+      </c>
+      <c r="N1" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="O1" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="P1" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="Q1" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="R1" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="S1" t="s" s="0">
+        <v>62</v>
       </c>
     </row>
     <row r="2">
@@ -629,37 +686,55 @@
         <v>16</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F2" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>58</v>
+        <v>65</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>60</v>
-      </c>
-      <c r="L2" t="b" s="0">
-        <v>0</v>
-      </c>
-      <c r="M2" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="N2" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="O2" t="b" s="0">
         <v>1</v>
+      </c>
+      <c r="P2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R2" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S2" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="3">
@@ -670,37 +745,55 @@
         <v>16</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="F3" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J3" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K3" t="s" s="0">
-        <v>63</v>
-      </c>
-      <c r="L3" t="b" s="0">
-        <v>1</v>
-      </c>
-      <c r="M3" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="N3" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="O3" t="b" s="0">
         <v>0</v>
+      </c>
+      <c r="P3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R3" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S3" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="4">
@@ -711,37 +804,55 @@
         <v>19</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F4" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>57</v>
-      </c>
-      <c r="J4" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
+      </c>
+      <c r="J4" t="n" s="0">
+        <v>5.0</v>
       </c>
       <c r="K4" t="s" s="0">
-        <v>67</v>
-      </c>
-      <c r="L4" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L4" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M4" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="N4" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="O4" t="b" s="0">
         <v>0</v>
       </c>
-      <c r="M4" t="b" s="0">
-        <v>0</v>
+      <c r="P4" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q4" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R4" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S4" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="5">
@@ -752,37 +863,55 @@
         <v>19</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F5" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="J5" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>72</v>
-      </c>
-      <c r="L5" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="N5" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="O5" t="b" s="0">
         <v>0</v>
       </c>
-      <c r="M5" t="b" s="0">
-        <v>0</v>
+      <c r="P5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R5" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S5" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="6">
@@ -793,37 +922,55 @@
         <v>22</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F6" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>75</v>
-      </c>
-      <c r="L6" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="N6" t="s" s="0">
+        <v>82</v>
+      </c>
+      <c r="O6" t="b" s="0">
         <v>0</v>
       </c>
-      <c r="M6" t="b" s="0">
-        <v>0</v>
+      <c r="P6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R6" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S6" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
     <row r="7">
@@ -834,37 +981,55 @@
         <v>25</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="F7" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>79</v>
-      </c>
-      <c r="L7" t="b" s="0">
+        <v>64</v>
+      </c>
+      <c r="L7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="M7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="N7" t="s" s="0">
+        <v>86</v>
+      </c>
+      <c r="O7" t="b" s="0">
         <v>0</v>
       </c>
-      <c r="M7" t="b" s="0">
-        <v>0</v>
+      <c r="P7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="Q7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="R7" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="S7" t="s" s="0">
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance Maturity Model Service and Excel Integration
- Added validation methods in MaturityModelService to ensure data integrity during model preparation.
- Introduced MaturityModelExcelPersistenceIntegrationTest to verify the export, edit, and import workflow of maturity models using Excel.
- Updated MaturityModelExcelServiceTest to include new headers in exported sheets and adjusted the official template model to reflect changes in scoring configurations.
- Created MaturityModelExcelWorkflowTest to validate the entire lifecycle of maturity models, including export, import, and editing functionalities.
- Modified error handling in useMaturityModelEditor hook to improve user feedback during workbook loading.
- Updated maturity model template to align with new export headers and functionalities.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/maturity-model-template.xlsx
+++ b/frontend/public/templates/maturity-model-template.xlsx
@@ -12,12 +12,13 @@
     <sheet name="Modules" r:id="rId6" sheetId="4"/>
     <sheet name="Practices" r:id="rId7" sheetId="5"/>
     <sheet name="Questions" r:id="rId8" sheetId="6"/>
+    <sheet name="Instructions" r:id="rId9" sheetId="7"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="141">
   <si>
     <t>modelName</t>
   </si>
@@ -28,36 +29,87 @@
     <t>modelAutoEvaluated</t>
   </si>
   <si>
+    <t>modelAggregationRule</t>
+  </si>
+  <si>
+    <t>modelChangelogMarkdown</t>
+  </si>
+  <si>
     <t>Your Maturity Model Name</t>
   </si>
   <si>
     <t>Description of what this maturity model assesses</t>
   </si>
   <si>
+    <t>WEIGHTED_AVERAGE</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
     <t>number</t>
   </si>
   <si>
     <t>name</t>
   </si>
   <si>
+    <t>description</t>
+  </si>
+  <si>
+    <t>Not Implemented</t>
+  </si>
+  <si>
+    <t>Initial</t>
+  </si>
+  <si>
+    <t>Managed</t>
+  </si>
+  <si>
+    <t>Defined</t>
+  </si>
+  <si>
+    <t>Optimised</t>
+  </si>
+  <si>
     <t>dimensionId</t>
   </si>
   <si>
     <t>dimensionName</t>
   </si>
   <si>
+    <t>dimensionDescription</t>
+  </si>
+  <si>
+    <t>dimensionWeight</t>
+  </si>
+  <si>
+    <t>dimensionAggregationRule</t>
+  </si>
+  <si>
+    <t>dimensionMappingRules</t>
+  </si>
+  <si>
+    <t>dimensionGatingRules</t>
+  </si>
+  <si>
     <t>dimension_1</t>
   </si>
   <si>
     <t>Process Management</t>
   </si>
   <si>
+    <t>How well processes are defined and managed</t>
+  </si>
+  <si>
     <t>dimension_2</t>
   </si>
   <si>
     <t>Quality Assurance</t>
   </si>
   <si>
+    <t>Quality control and assurance practices</t>
+  </si>
+  <si>
     <t>moduleCode</t>
   </si>
   <si>
@@ -67,6 +119,15 @@
     <t>moduleDescription</t>
   </si>
   <si>
+    <t>moduleWeight</t>
+  </si>
+  <si>
+    <t>moduleAggregationRule</t>
+  </si>
+  <si>
+    <t>moduleGatingRules</t>
+  </si>
+  <si>
     <t>PM_CORE</t>
   </si>
   <si>
@@ -115,6 +176,15 @@
     <t>practiceRequiresEvidence</t>
   </si>
   <si>
+    <t>practiceWeight</t>
+  </si>
+  <si>
+    <t>practiceAggregationRule</t>
+  </si>
+  <si>
+    <t>practiceGatingRules</t>
+  </si>
+  <si>
     <t>P1_PD</t>
   </si>
   <si>
@@ -208,12 +278,12 @@
     <t>questionRanges</t>
   </si>
   <si>
+    <t>questionBooleanCorrectAnswer</t>
+  </si>
+  <si>
     <t>Q1_APD</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>Are processes documented?</t>
   </si>
   <si>
@@ -223,6 +293,9 @@
     <t>Check if there are written process descriptions</t>
   </si>
   <si>
+    <t>true</t>
+  </si>
+  <si>
     <t>Q2_ITADPO</t>
   </si>
   <si>
@@ -241,7 +314,13 @@
     <t>likert</t>
   </si>
   <si>
-    <t>Rate on your model maturity scale (1 = lowest).</t>
+    <t>Never</t>
+  </si>
+  <si>
+    <t>Always</t>
+  </si>
+  <si>
+    <t>Rate from 1 (never) to 7 (always).</t>
   </si>
   <si>
     <t>Q4_WMLBDTP</t>
@@ -256,7 +335,7 @@
     <t>[{"label":"Initial / ad-hoc","score":0.0,"rawValue":null},{"label":"Repeatable","score":0.25,"rawValue":null},{"label":"Defined","score":0.5,"rawValue":null},{"label":"Managed","score":0.75,"rawValue":null},{"label":"Optimizing","score":1.0,"rawValue":null}]</t>
   </si>
   <si>
-    <t>Each option maps to a level number on your scale. Use JSON: array of {label level}.</t>
+    <t>Choose one option. Each option has a normalized score between 0 and 1.</t>
   </si>
   <si>
     <t>Q5_AQSD</t>
@@ -278,6 +357,90 @@
   </si>
   <si>
     <t>Provide details about ongoing quality improvements</t>
+  </si>
+  <si>
+    <t>Q7_ISSUES</t>
+  </si>
+  <si>
+    <t>How many unresolved quality issues remain?</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>Fewer issues produce a higher score.</t>
+  </si>
+  <si>
+    <t>Q8_REVIEWED</t>
+  </si>
+  <si>
+    <t>What percentage of processes are reviewed?</t>
+  </si>
+  <si>
+    <t>percentage</t>
+  </si>
+  <si>
+    <t>Enter an integer percentage from 0 to 100.</t>
+  </si>
+  <si>
+    <t>Q9_CONTROLS</t>
+  </si>
+  <si>
+    <t>Which quality controls are in place?</t>
+  </si>
+  <si>
+    <t>multiple_selection</t>
+  </si>
+  <si>
+    <t>[{"label":"Documented controls","score":null,"rawValue":2.0},{"label":"Regular audits","score":null,"rawValue":3.0}]</t>
+  </si>
+  <si>
+    <t>Select all that apply; selected raw values are added.</t>
+  </si>
+  <si>
+    <t>Edit data on the six model sheets; keep their names and column headers. Optional newer columns may be omitted in older workbooks.</t>
+  </si>
+  <si>
+    <t>Use one row on Model. Imported models are inactive; choose a domain in the editor and review before saving as a new model or version.</t>
+  </si>
+  <si>
+    <t>Levels: define 2 to 12 levels numbered 1..N. Description is optional.</t>
+  </si>
+  <si>
+    <t>Join items using dimensionId, moduleCode and practiceCode. Codes must be unique among siblings. If changing a code, update all child references, dependencies and gating rules.</t>
+  </si>
+  <si>
+    <t>Sheet row order determines dimension, module, practice and question order. Every dimension/module/practice must lead to a question. Remove child rows when deleting an item.</t>
+  </si>
+  <si>
+    <t>Aggregation rules: AVERAGE, WEIGHTED_AVERAGE, MINIMUM, MAXIMUM, SUM, MEDIAN. Empty values use the application defaults. Weights must be positive.</t>
+  </si>
+  <si>
+    <t>dimensionMappingRules: JSON array, one threshold per level, starting at zero, strictly increasing within 0..1. Example: [{"levelNumber":1,"minimumScore":0},{"levelNumber":2,"minimumScore":0.5}].</t>
+  </si>
+  <si>
+    <t>Gating rules: JSON array. Example: [{"order":0,"selection":"specificChild","childCode":"Q1","operator":"&lt;","threshold":0.5,"operation":"set","value":0}]. Reference immediate child codes. selection: specificChild/anyChild/allChildren; operator: &lt;, &lt;=, ==, &gt;=, &gt;; operation: set/add/subtract.</t>
+  </si>
+  <si>
+    <t>Question types: boolean, likert, open_answer, multiple_choice, multiple_selection, numeric, percentage. Leave type-specific columns empty for other types.</t>
+  </si>
+  <si>
+    <t>boolean: questionBooleanCorrectAnswer is true or false (default true). practiceRequiresEvidence and questionRequired also use true/false.</t>
+  </si>
+  <si>
+    <t>multiple_choice questionChoices: [{"label":"No","score":0},{"label":"Yes","score":1}]. Scores are between 0 and 1.</t>
+  </si>
+  <si>
+    <t>multiple_selection questionChoices: [{"label":"Control A","rawValue":2},{"label":"Control B","rawValue":3}]. Raw values are nonnegative and their total must be positive.</t>
+  </si>
+  <si>
+    <t>likert: questionScalePointCount is 2..100; optional endpoint labels are at most 50 characters; questionScaleHighPointIsMaximum controls direction.</t>
+  </si>
+  <si>
+    <t>numeric/percentage: integer questionRangeMin &lt; questionRangeMax; questionRangeHighValueIsMaximum controls direction. questionRanges is a legacy JSON format; keep it blank when using bounds.</t>
+  </si>
+  <si>
+    <t>dependsOnQuestionCode must refer to a boolean question in the same practice. Leave blank for independent questions.</t>
   </si>
 </sst>
 </file>
@@ -322,7 +485,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -335,16 +498,28 @@
       <c r="C1" t="s" s="0">
         <v>2</v>
       </c>
+      <c r="D1" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>4</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C2" t="b" s="0">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -354,15 +529,73 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>6</v>
+        <v>10</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>2.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -372,31 +605,76 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:G3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>8</v>
+        <v>18</v>
+      </c>
+      <c r="C1" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>23</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>10</v>
+        <v>25</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="D2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>12</v>
+        <v>28</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="D3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -406,77 +684,122 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>15</v>
+        <v>32</v>
+      </c>
+      <c r="E1" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="F1" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>35</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>18</v>
+        <v>38</v>
+      </c>
+      <c r="E2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G2" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>21</v>
+        <v>41</v>
+      </c>
+      <c r="E3" t="n" s="0">
+        <v>1.5</v>
+      </c>
+      <c r="F3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G3" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>23</v>
+        <v>43</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>24</v>
+        <v>44</v>
+      </c>
+      <c r="E4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G4" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>27</v>
+        <v>47</v>
+      </c>
+      <c r="E5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="F5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -486,127 +809,181 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>31</v>
+        <v>51</v>
+      </c>
+      <c r="G1" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="H1" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="I1" t="s" s="0">
+        <v>54</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>33</v>
+        <v>56</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="F2" t="b" s="0">
         <v>0</v>
       </c>
+      <c r="G2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I2" t="s" s="0">
+        <v>8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="F3" t="b" s="0">
         <v>0</v>
       </c>
+      <c r="G3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I3" t="s" s="0">
+        <v>8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>39</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>40</v>
+        <v>63</v>
       </c>
       <c r="F4" t="b" s="0">
         <v>0</v>
       </c>
+      <c r="G4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I4" t="s" s="0">
+        <v>8</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>42</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>43</v>
+        <v>66</v>
       </c>
       <c r="F5" t="b" s="0">
         <v>0</v>
       </c>
+      <c r="G5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I5" t="s" s="0">
+        <v>8</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>46</v>
+        <v>69</v>
       </c>
       <c r="F6" t="b" s="0">
         <v>0</v>
+      </c>
+      <c r="G6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="I6" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -616,420 +993,715 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:S7"/>
+  <dimension ref="A1:T10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="B1" t="s" s="0">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C1" t="s" s="0">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="D1" t="s" s="0">
-        <v>47</v>
+        <v>70</v>
       </c>
       <c r="E1" t="s" s="0">
-        <v>48</v>
+        <v>71</v>
       </c>
       <c r="F1" t="s" s="0">
-        <v>49</v>
+        <v>72</v>
       </c>
       <c r="G1" t="s" s="0">
-        <v>50</v>
+        <v>73</v>
       </c>
       <c r="H1" t="s" s="0">
-        <v>51</v>
+        <v>74</v>
       </c>
       <c r="I1" t="s" s="0">
-        <v>52</v>
+        <v>75</v>
       </c>
       <c r="J1" t="s" s="0">
-        <v>53</v>
+        <v>76</v>
       </c>
       <c r="K1" t="s" s="0">
-        <v>54</v>
+        <v>77</v>
       </c>
       <c r="L1" t="s" s="0">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="M1" t="s" s="0">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="N1" t="s" s="0">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="O1" t="s" s="0">
-        <v>58</v>
+        <v>81</v>
       </c>
       <c r="P1" t="s" s="0">
-        <v>59</v>
+        <v>82</v>
       </c>
       <c r="Q1" t="s" s="0">
-        <v>60</v>
+        <v>83</v>
       </c>
       <c r="R1" t="s" s="0">
-        <v>61</v>
+        <v>84</v>
       </c>
       <c r="S1" t="s" s="0">
-        <v>62</v>
+        <v>85</v>
+      </c>
+      <c r="T1" t="s" s="0">
+        <v>86</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F2" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>65</v>
+        <v>88</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="I2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="J2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="K2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="M2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>67</v>
+        <v>90</v>
       </c>
       <c r="O2" t="b" s="0">
         <v>1</v>
       </c>
       <c r="P2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S2" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T2" t="s" s="0">
+        <v>91</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>16</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>32</v>
+        <v>55</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F3" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>69</v>
+        <v>93</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="I3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="J3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="K3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="M3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>70</v>
+        <v>94</v>
       </c>
       <c r="O3" t="b" s="0">
         <v>0</v>
       </c>
       <c r="P3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S3" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T3" t="s" s="0">
+        <v>91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>71</v>
+        <v>95</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F4" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>72</v>
+        <v>96</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>73</v>
+        <v>97</v>
       </c>
       <c r="I4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="J4" t="n" s="0">
-        <v>5.0</v>
+        <v>7.0</v>
       </c>
       <c r="K4" t="s" s="0">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>64</v>
+        <v>99</v>
       </c>
       <c r="M4" t="b" s="0">
         <v>1</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>74</v>
+        <v>100</v>
       </c>
       <c r="O4" t="b" s="0">
         <v>0</v>
       </c>
       <c r="P4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S4" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T4" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>75</v>
+        <v>101</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>76</v>
+        <v>102</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>77</v>
+        <v>103</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="J5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="K5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="M5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>79</v>
+        <v>105</v>
       </c>
       <c r="O5" t="b" s="0">
         <v>0</v>
       </c>
       <c r="P5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S5" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T5" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>41</v>
+        <v>64</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F6" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>66</v>
+        <v>89</v>
       </c>
       <c r="I6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="J6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="K6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="M6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="O6" t="b" s="0">
         <v>0</v>
       </c>
       <c r="P6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S6" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T6" t="s" s="0">
+        <v>91</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>44</v>
+        <v>67</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>84</v>
+        <v>110</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>85</v>
+        <v>111</v>
       </c>
       <c r="I7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="J7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="K7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="L7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="M7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="O7" t="b" s="0">
         <v>0</v>
       </c>
       <c r="P7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="Q7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="R7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="S7" t="s" s="0">
-        <v>64</v>
+        <v>8</v>
+      </c>
+      <c r="T7" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>113</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>114</v>
+      </c>
+      <c r="H8" t="s" s="0">
+        <v>115</v>
+      </c>
+      <c r="I8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="J8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="K8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="L8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="M8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="N8" t="s" s="0">
+        <v>116</v>
+      </c>
+      <c r="O8" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="P8" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="Q8" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="R8" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="S8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="T8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>117</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="G9" t="s" s="0">
+        <v>118</v>
+      </c>
+      <c r="H9" t="s" s="0">
+        <v>119</v>
+      </c>
+      <c r="I9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="J9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="K9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="L9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="M9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="N9" t="s" s="0">
+        <v>120</v>
+      </c>
+      <c r="O9" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="P9" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="Q9" t="n" s="0">
+        <v>100.0</v>
+      </c>
+      <c r="R9" t="b" s="0">
+        <v>1</v>
+      </c>
+      <c r="S9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="T9" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>121</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="F10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="G10" t="s" s="0">
+        <v>122</v>
+      </c>
+      <c r="H10" t="s" s="0">
+        <v>123</v>
+      </c>
+      <c r="I10" t="s" s="0">
+        <v>124</v>
+      </c>
+      <c r="J10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="K10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="L10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="M10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="N10" t="s" s="0">
+        <v>125</v>
+      </c>
+      <c r="O10" t="b" s="0">
+        <v>0</v>
+      </c>
+      <c r="P10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="Q10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="R10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="S10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="T10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:A15"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="1" max="1" width="120.0" customWidth="true"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: add question dependency conditions and related functionality
- Introduced a new column `dependency_condition` in the `questions` table to store conditions for question dependencies.
- Implemented logic to update dependency conditions based on parent question types (boolean, multiple choice).
- Created a new service `QuestionDependenciesTest` to validate dependency conditions and their activation logic.
- Added migration scripts to ensure existing data is preserved and correctly migrated to the new structure.
- Developed frontend components for managing question dependencies, including a new `QuestionDependencyField`.
- Enhanced the question editor to support dependency conditions with appropriate UI elements and validation.
- Added comprehensive tests for dependency matching and validation logic, ensuring robust functionality.
- Documented the new feature in `question-dependency-conditions.md` for clarity on usage and implementation.
</commit_message>
<xml_diff>
--- a/frontend/public/templates/maturity-model-template.xlsx
+++ b/frontend/public/templates/maturity-model-template.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="144">
   <si>
     <t>modelName</t>
   </si>
@@ -281,6 +281,9 @@
     <t>questionBooleanCorrectAnswer</t>
   </si>
   <si>
+    <t>dependencyCondition</t>
+  </si>
+  <si>
     <t>Q1_APD</t>
   </si>
   <si>
@@ -305,6 +308,9 @@
     <t>Is someone specifically responsible for this process?</t>
   </si>
   <si>
+    <t>{"type":"boolean","answers":[true]}</t>
+  </si>
+  <si>
     <t>Q3_APMCAA</t>
   </si>
   <si>
@@ -332,7 +338,7 @@
     <t>multiple_choice</t>
   </si>
   <si>
-    <t>[{"label":"Initial / ad-hoc","score":0.0,"rawValue":null},{"label":"Repeatable","score":0.25,"rawValue":null},{"label":"Defined","score":0.5,"rawValue":null},{"label":"Managed","score":0.75,"rawValue":null},{"label":"Optimizing","score":1.0,"rawValue":null}]</t>
+    <t>[{"id":"83b8ced5-fd57-43bc-877c-4446972332bb","label":"Initial / ad-hoc","score":0.0,"rawValue":null},{"id":"eba88088-51aa-4019-9182-2b65d1266b08","label":"Repeatable","score":0.25,"rawValue":null},{"id":"811667b1-f494-48c2-943b-c1ad66e6d9ca","label":"Defined","score":0.5,"rawValue":null},{"id":"f600418b-6b1d-4c41-8335-d191e3f79dfb","label":"Managed","score":0.75,"rawValue":null},{"id":"996f3142-e358-4de9-8312-1f7928908f6d","label":"Optimizing","score":1.0,"rawValue":null}]</t>
   </si>
   <si>
     <t>Choose one option. Each option has a normalized score between 0 and 1.</t>
@@ -392,7 +398,7 @@
     <t>multiple_selection</t>
   </si>
   <si>
-    <t>[{"label":"Documented controls","score":null,"rawValue":2.0},{"label":"Regular audits","score":null,"rawValue":3.0}]</t>
+    <t>[{"id":null,"label":"Documented controls","score":null,"rawValue":2.0},{"id":null,"label":"Regular audits","score":null,"rawValue":3.0}]</t>
   </si>
   <si>
     <t>Select all that apply; selected raw values are added.</t>
@@ -413,7 +419,7 @@
     <t>Sheet row order determines dimension, module, practice and question order. Every dimension/module/practice must lead to a question. Remove child rows when deleting an item.</t>
   </si>
   <si>
-    <t>Aggregation rules: AVERAGE, WEIGHTED_AVERAGE, MINIMUM, MAXIMUM, SUM, MEDIAN. Empty values use the application defaults. Weights must be positive.</t>
+    <t>Aggregation rules: AVERAGE, WEIGHTED_AVERAGE, MINIMUM, MAXIMUM, SUM, MEDIAN. Empty values use the application defaults. Weights must be positive; optional questions may have zero weight.</t>
   </si>
   <si>
     <t>dimensionMappingRules: JSON array, one threshold per level, starting at zero, strictly increasing within 0..1. Example: [{"levelNumber":1,"minimumScore":0},{"levelNumber":2,"minimumScore":0.5}].</t>
@@ -440,7 +446,10 @@
     <t>numeric/percentage: integer questionRangeMin &lt; questionRangeMax; questionRangeHighValueIsMaximum controls direction. questionRanges is a legacy JSON format; keep it blank when using bounds.</t>
   </si>
   <si>
-    <t>dependsOnQuestionCode must refer to a boolean question in the same practice. Leave blank for independent questions.</t>
+    <t>dependencyCondition JSON examples: {"type":"boolean","answers":[false]}, {"type":"multiple_choice","optionIds":["option-a"]}, {"type":"likert","points":[3,4,5]}. Select one or more answers; any selected answer activates the question. Preserve choice id values when editing options.</t>
+  </si>
+  <si>
+    <t>dependsOnQuestionCode must refer to a Yes / No, Multiple choice, or Scale question in the same practice. dependencyCondition specifies matching answers; a legacy boolean dependency defaults to Yes.</t>
   </si>
 </sst>
 </file>
@@ -993,7 +1002,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:T10"/>
+  <dimension ref="A1:U10"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -1057,6 +1066,9 @@
       <c r="T1" t="s" s="0">
         <v>86</v>
       </c>
+      <c r="U1" t="s" s="0">
+        <v>87</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
@@ -1069,7 +1081,7 @@
         <v>55</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>8</v>
@@ -1078,10 +1090,10 @@
         <v>1.0</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H2" t="s" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I2" t="s" s="0">
         <v>8</v>
@@ -1099,7 +1111,7 @@
         <v>8</v>
       </c>
       <c r="N2" t="s" s="0">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O2" t="b" s="0">
         <v>1</v>
@@ -1117,7 +1129,10 @@
         <v>8</v>
       </c>
       <c r="T2" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="U2" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="3">
@@ -1131,19 +1146,19 @@
         <v>55</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="F3" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H3" t="s" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I3" t="s" s="0">
         <v>8</v>
@@ -1161,7 +1176,7 @@
         <v>8</v>
       </c>
       <c r="N3" t="s" s="0">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="O3" t="b" s="0">
         <v>0</v>
@@ -1179,7 +1194,10 @@
         <v>8</v>
       </c>
       <c r="T3" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="U3" t="s" s="0">
+        <v>96</v>
       </c>
     </row>
     <row r="4">
@@ -1193,7 +1211,7 @@
         <v>58</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>8</v>
@@ -1202,10 +1220,10 @@
         <v>1.0</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H4" t="s" s="0">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="I4" t="s" s="0">
         <v>8</v>
@@ -1214,16 +1232,16 @@
         <v>7.0</v>
       </c>
       <c r="K4" t="s" s="0">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="L4" t="s" s="0">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="M4" t="b" s="0">
         <v>1</v>
       </c>
       <c r="N4" t="s" s="0">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="O4" t="b" s="0">
         <v>0</v>
@@ -1241,6 +1259,9 @@
         <v>8</v>
       </c>
       <c r="T4" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U4" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1255,7 +1276,7 @@
         <v>61</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>8</v>
@@ -1264,13 +1285,13 @@
         <v>1.0</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H5" t="s" s="0">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="I5" t="s" s="0">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="J5" t="s" s="0">
         <v>8</v>
@@ -1285,7 +1306,7 @@
         <v>8</v>
       </c>
       <c r="N5" t="s" s="0">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="O5" t="b" s="0">
         <v>0</v>
@@ -1303,6 +1324,9 @@
         <v>8</v>
       </c>
       <c r="T5" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U5" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1317,7 +1341,7 @@
         <v>64</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>8</v>
@@ -1326,10 +1350,10 @@
         <v>1.0</v>
       </c>
       <c r="G6" t="s" s="0">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H6" t="s" s="0">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="I6" t="s" s="0">
         <v>8</v>
@@ -1347,7 +1371,7 @@
         <v>8</v>
       </c>
       <c r="N6" t="s" s="0">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="O6" t="b" s="0">
         <v>0</v>
@@ -1365,7 +1389,10 @@
         <v>8</v>
       </c>
       <c r="T6" t="s" s="0">
-        <v>91</v>
+        <v>92</v>
+      </c>
+      <c r="U6" t="s" s="0">
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -1379,7 +1406,7 @@
         <v>67</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>8</v>
@@ -1388,10 +1415,10 @@
         <v>1.0</v>
       </c>
       <c r="G7" t="s" s="0">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H7" t="s" s="0">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I7" t="s" s="0">
         <v>8</v>
@@ -1409,7 +1436,7 @@
         <v>8</v>
       </c>
       <c r="N7" t="s" s="0">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="O7" t="b" s="0">
         <v>0</v>
@@ -1427,6 +1454,9 @@
         <v>8</v>
       </c>
       <c r="T7" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U7" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1441,7 +1471,7 @@
         <v>67</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>8</v>
@@ -1450,10 +1480,10 @@
         <v>1.0</v>
       </c>
       <c r="G8" t="s" s="0">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H8" t="s" s="0">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>8</v>
@@ -1471,7 +1501,7 @@
         <v>8</v>
       </c>
       <c r="N8" t="s" s="0">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="O8" t="b" s="0">
         <v>1</v>
@@ -1489,6 +1519,9 @@
         <v>8</v>
       </c>
       <c r="T8" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U8" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1503,7 +1536,7 @@
         <v>67</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>8</v>
@@ -1512,10 +1545,10 @@
         <v>1.0</v>
       </c>
       <c r="G9" t="s" s="0">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H9" t="s" s="0">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>8</v>
@@ -1533,7 +1566,7 @@
         <v>8</v>
       </c>
       <c r="N9" t="s" s="0">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="O9" t="b" s="0">
         <v>1</v>
@@ -1551,6 +1584,9 @@
         <v>8</v>
       </c>
       <c r="T9" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U9" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1565,7 +1601,7 @@
         <v>67</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>8</v>
@@ -1574,13 +1610,13 @@
         <v>1.0</v>
       </c>
       <c r="G10" t="s" s="0">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H10" t="s" s="0">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="I10" t="s" s="0">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="J10" t="s" s="0">
         <v>8</v>
@@ -1595,7 +1631,7 @@
         <v>8</v>
       </c>
       <c r="N10" t="s" s="0">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="O10" t="b" s="0">
         <v>0</v>
@@ -1613,6 +1649,9 @@
         <v>8</v>
       </c>
       <c r="T10" t="s" s="0">
+        <v>8</v>
+      </c>
+      <c r="U10" t="s" s="0">
         <v>8</v>
       </c>
     </row>
@@ -1623,7 +1662,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="120.0" customWidth="true"/>
@@ -1631,77 +1670,82 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s" s="0">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s" s="0">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="0">
-        <v>128</v>
+        <v>130</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>132</v>
+        <v>134</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>133</v>
+        <v>135</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>134</v>
+        <v>136</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
-        <v>135</v>
+        <v>137</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="0">
-        <v>136</v>
+        <v>138</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="0">
-        <v>137</v>
+        <v>139</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>138</v>
+        <v>140</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="0">
-        <v>140</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>143</v>
       </c>
     </row>
   </sheetData>

</xml_diff>